<commit_message>
test/[Product Display - Shopping Cart] add test cases for Req id SRS-FN-Product-008 on ProductDisplay_TestCases File and fix misunderstand for subtotal and total calculations
</commit_message>
<xml_diff>
--- a/TestCases_Docs/ProductDisplay_TestCases.xlsx
+++ b/TestCases_Docs/ProductDisplay_TestCases.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenovo\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\iti\QA\Clothing-Web-Portal\TestCases_Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9476313-963C-4400-A863-8CB054D8C28B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45992F72-873E-47AB-8CC7-8699CBC14988}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11520" yWindow="0" windowWidth="11520" windowHeight="12360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="11520" windowHeight="12360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Product Test Cases" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="302">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="307">
   <si>
     <t>TesTCASE ID</t>
   </si>
@@ -1346,6 +1346,23 @@
   </si>
   <si>
     <t>SRS-FN-Product-007</t>
+  </si>
+  <si>
+    <t>TC_Product_010</t>
+  </si>
+  <si>
+    <t>Verify UI elements for the supplier name of the products are displayed</t>
+  </si>
+  <si>
+    <t>1. Open website
+2. Navigate to products page
+3. Observe UI elements for the supplier name of the products are displayed</t>
+  </si>
+  <si>
+    <t>supplier name is displayed</t>
+  </si>
+  <si>
+    <t>SRS-FN-Product-008</t>
   </si>
 </sst>
 </file>
@@ -1522,7 +1539,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1665,11 +1682,6 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1907,12 +1919,10 @@
     <col min="10" max="10" width="18.21875" customWidth="1"/>
     <col min="11" max="11" width="16.6640625" customWidth="1"/>
     <col min="12" max="12" width="33.33203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="15" width="18.21875" customWidth="1"/>
-    <col min="16" max="27" width="18.21875" style="54" customWidth="1"/>
-    <col min="28" max="16384" width="12.6640625" style="54"/>
+    <col min="13" max="27" width="18.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:27" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="37" t="s">
         <v>0</v>
       </c>
@@ -1959,7 +1969,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:27" customFormat="1" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:27" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="38" t="s">
         <v>251</v>
       </c>
@@ -2010,7 +2020,7 @@
       <c r="Z2" s="2"/>
       <c r="AA2" s="2"/>
     </row>
-    <row r="3" spans="1:27" customFormat="1" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:27" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="38" t="s">
         <v>252</v>
       </c>
@@ -2059,7 +2069,7 @@
       <c r="Z3" s="2"/>
       <c r="AA3" s="2"/>
     </row>
-    <row r="4" spans="1:27" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:27" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A4" s="38" t="s">
         <v>253</v>
       </c>
@@ -2108,7 +2118,7 @@
       <c r="Z4" s="2"/>
       <c r="AA4" s="2"/>
     </row>
-    <row r="5" spans="1:27" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:27" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A5" s="38" t="s">
         <v>254</v>
       </c>
@@ -2126,7 +2136,7 @@
         <v>278</v>
       </c>
       <c r="G5" s="41"/>
-      <c r="H5" s="56" t="s">
+      <c r="H5" s="53" t="s">
         <v>288</v>
       </c>
       <c r="I5" s="38"/>
@@ -2157,7 +2167,7 @@
       <c r="Z5" s="2"/>
       <c r="AA5" s="2"/>
     </row>
-    <row r="6" spans="1:27" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="38" t="s">
         <v>264</v>
       </c>
@@ -2194,7 +2204,7 @@
       </c>
       <c r="O6" s="44"/>
     </row>
-    <row r="7" spans="1:27" customFormat="1" ht="51.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:27" ht="51.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="38" t="s">
         <v>265</v>
       </c>
@@ -2269,18 +2279,18 @@
         <v>293</v>
       </c>
       <c r="O8" s="48"/>
-      <c r="P8" s="55"/>
-      <c r="Q8" s="55"/>
-      <c r="R8" s="55"/>
-      <c r="S8" s="55"/>
-      <c r="T8" s="55"/>
-      <c r="U8" s="55"/>
-      <c r="V8" s="55"/>
-      <c r="W8" s="55"/>
-      <c r="X8" s="55"/>
-      <c r="Y8" s="55"/>
-      <c r="Z8" s="55"/>
-      <c r="AA8" s="55"/>
+      <c r="P8" s="20"/>
+      <c r="Q8" s="20"/>
+      <c r="R8" s="20"/>
+      <c r="S8" s="20"/>
+      <c r="T8" s="20"/>
+      <c r="U8" s="20"/>
+      <c r="V8" s="20"/>
+      <c r="W8" s="20"/>
+      <c r="X8" s="20"/>
+      <c r="Y8" s="20"/>
+      <c r="Z8" s="20"/>
+      <c r="AA8" s="20"/>
     </row>
     <row r="9" spans="1:27" ht="52.8" x14ac:dyDescent="0.25">
       <c r="A9" s="38" t="s">
@@ -2357,23 +2367,67 @@
         <v>293</v>
       </c>
       <c r="O10" s="45"/>
-      <c r="P10" s="53"/>
-      <c r="Q10" s="53"/>
-      <c r="R10" s="53"/>
-      <c r="S10" s="53"/>
-      <c r="T10" s="53"/>
-      <c r="U10" s="53"/>
-      <c r="V10" s="53"/>
-      <c r="W10" s="53"/>
-      <c r="X10" s="53"/>
-      <c r="Y10" s="53"/>
-      <c r="Z10" s="53"/>
-      <c r="AA10" s="53"/>
-    </row>
-    <row r="11" spans="1:27" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="H11" s="13"/>
-      <c r="L11" s="13"/>
-      <c r="N11" s="13"/>
+      <c r="P10" s="14"/>
+      <c r="Q10" s="14"/>
+      <c r="R10" s="14"/>
+      <c r="S10" s="14"/>
+      <c r="T10" s="14"/>
+      <c r="U10" s="14"/>
+      <c r="V10" s="14"/>
+      <c r="W10" s="14"/>
+      <c r="X10" s="14"/>
+      <c r="Y10" s="14"/>
+      <c r="Z10" s="14"/>
+      <c r="AA10" s="14"/>
+    </row>
+    <row r="11" spans="1:27" ht="92.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="38" t="s">
+        <v>302</v>
+      </c>
+      <c r="B11" s="51" t="s">
+        <v>303</v>
+      </c>
+      <c r="C11" s="38" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" s="39" t="s">
+        <v>255</v>
+      </c>
+      <c r="E11" s="45"/>
+      <c r="F11" s="52" t="s">
+        <v>304</v>
+      </c>
+      <c r="G11" s="45"/>
+      <c r="H11" s="46" t="s">
+        <v>305</v>
+      </c>
+      <c r="I11" s="45"/>
+      <c r="J11" s="40" t="s">
+        <v>292</v>
+      </c>
+      <c r="K11" s="45"/>
+      <c r="L11" s="38" t="s">
+        <v>306</v>
+      </c>
+      <c r="M11" s="40" t="s">
+        <v>294</v>
+      </c>
+      <c r="N11" s="38" t="s">
+        <v>293</v>
+      </c>
+      <c r="O11" s="45"/>
+      <c r="P11" s="14"/>
+      <c r="Q11" s="14"/>
+      <c r="R11" s="14"/>
+      <c r="S11" s="14"/>
+      <c r="T11" s="14"/>
+      <c r="U11" s="14"/>
+      <c r="V11" s="14"/>
+      <c r="W11" s="14"/>
+      <c r="X11" s="14"/>
+      <c r="Y11" s="14"/>
+      <c r="Z11" s="14"/>
+      <c r="AA11" s="14"/>
     </row>
     <row r="12" spans="1:27" ht="13.2" x14ac:dyDescent="0.25">
       <c r="H12" s="13"/>
@@ -5553,7 +5607,7 @@
   </sheetData>
   <phoneticPr fontId="11" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C10" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C11" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"valid,invalid"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
test/Updated Product display Test Cases
</commit_message>
<xml_diff>
--- a/TestCases_Docs/ProductDisplay_TestCases.xlsx
+++ b/TestCases_Docs/ProductDisplay_TestCases.xlsx
@@ -162,7 +162,7 @@
 3. Observe stock status for each product</t>
   </si>
   <si>
-    <t>Stock status shows "In Stock: [n] units", "Low Stock", or "Out of Stock"</t>
+    <t>Stock status shows "In Stock: [n] units" or "Out of Stock"</t>
   </si>
   <si>
     <t>SRS-FN-Product-005</t>
@@ -295,7 +295,7 @@
     <t>TC_Product_012</t>
   </si>
   <si>
-    <t>Verify Add to Cart button is disabled when product is Out of Stock.</t>
+    <t>Verify Add to Cart button is disappeared when product is Out of Stock.</t>
   </si>
   <si>
     <t>1.Client has a valid account
@@ -308,7 +308,7 @@
  4. Observe Add to Cart button</t>
   </si>
   <si>
-    <t>Add to Cart button is disabled (not clickable).</t>
+    <t>Add to Cart button is disappeared  and displays text "Out of stock".</t>
   </si>
   <si>
     <t>Functional</t>
@@ -370,7 +370,7 @@
    6. Navigate to Cart page</t>
   </si>
   <si>
-    <t>1. Success message appears   
+    <t>1. Success message :"Added to cart"
 2. Product appears in cart with correct quantity
  3. Cart total updates correctly</t>
   </si>
@@ -2143,7 +2143,7 @@
     <col customWidth="1" min="5" max="5" width="56.38"/>
     <col customWidth="1" min="6" max="6" width="78.13"/>
     <col customWidth="1" min="7" max="7" width="32.63"/>
-    <col customWidth="1" min="8" max="8" width="56.5"/>
+    <col customWidth="1" min="8" max="8" width="73.5"/>
     <col customWidth="1" min="9" max="9" width="29.5"/>
     <col customWidth="1" min="10" max="10" width="18.25"/>
     <col customWidth="1" min="11" max="11" width="16.63"/>

</xml_diff>